<commit_message>
feat: Update contact messages data file
</commit_message>
<xml_diff>
--- a/data/contact_messages.xlsx
+++ b/data/contact_messages.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,28 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>PACASAAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tessss</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>mamamo@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SADVDAVAVADVFSFBSF</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DFSFSBDFDFB</t>
         </is>
       </c>
     </row>

</xml_diff>